<commit_message>
Planilha de exemplo com nomes genéricos
</commit_message>
<xml_diff>
--- a/exemplos/planilha-import-exemplo.xlsx
+++ b/exemplos/planilha-import-exemplo.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brokers SMS | WHATSAPP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suporte Técnico" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fornecedores Antigos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fornecedores Externos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ferramentas Internas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arquivo Antigo" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -472,7 +472,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Brokers SMS | WHATSAPP</t>
+          <t>Mensageria</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -521,7 +521,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Brokers SMS | WHATSAPP</t>
+          <t>Mensageria</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Duplicado de teste — deve consolidar com Brokers</t>
+          <t>Duplicado de teste — deve consolidar com Fornecedores Externos</t>
         </is>
       </c>
     </row>

</xml_diff>